<commit_message>
Actualización: app.py, automatizacion_santamaria.py, historial_urls, Excel y nuevos archivos de diseño web
</commit_message>
<xml_diff>
--- a/El Tiempo.xlsx
+++ b/El Tiempo.xlsx
@@ -53,7 +53,7 @@
     <font>
       <name val="Century Gothic"/>
       <b val="1"/>
-      <color rgb="000D47A1"/>
+      <color rgb="004A148C"/>
       <sz val="11"/>
     </font>
     <font>
@@ -91,13 +91,49 @@
     <font>
       <name val="Century Gothic"/>
       <b val="1"/>
-      <color rgb="004A148C"/>
+      <color rgb="000D47A1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Century Gothic"/>
       <b val="1"/>
-      <color rgb="00880E4F"/>
+      <color rgb="0033691E"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Century Gothic"/>
+      <b val="1"/>
+      <color rgb="0000695C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Century Gothic"/>
+      <b val="1"/>
+      <color rgb="00E65100"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Century Gothic"/>
+      <b val="1"/>
+      <color rgb="00B71C1C"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Century Gothic"/>
+      <b val="1"/>
+      <color rgb="001B5E20"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Century Gothic"/>
+      <b val="1"/>
+      <color rgb="001565C0"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Century Gothic"/>
+      <b val="1"/>
+      <color rgb="0037474F"/>
       <sz val="11"/>
     </font>
     <font>
@@ -109,43 +145,7 @@
     <font>
       <name val="Century Gothic"/>
       <b val="1"/>
-      <color rgb="0033691E"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Century Gothic"/>
-      <b val="1"/>
-      <color rgb="0000695C"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Century Gothic"/>
-      <b val="1"/>
-      <color rgb="001565C0"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Century Gothic"/>
-      <b val="1"/>
-      <color rgb="00B71C1C"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Century Gothic"/>
-      <b val="1"/>
-      <color rgb="00E65100"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Century Gothic"/>
-      <b val="1"/>
-      <color rgb="0037474F"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Century Gothic"/>
-      <b val="1"/>
-      <color rgb="001B5E20"/>
+      <color rgb="00880E4F"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -273,16 +273,16 @@
     <xf numFmtId="0" fontId="16" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="19" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="20" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -754,32 +754,32 @@
       <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Estas son las cédulas que tienen que declarar renta está</t>
+          <t>Venezuela supera un año bajo excepción inconstitucional</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/economia/finanzas-personales/estas-son-las-cedulas-que-tienen-que-declarar-renta-esta-semana-del-18-al-21-de-agosto-3578997</t>
+          <t>https://www.eltiempo.com/mundo/venezuela/venezuela-suma-mas-de-un-ano-bajo-estado-de-excepcion-inconstitucional-la-acumulacion-de-competencias-del-ejecutivo-crecio-de-manera-exponencial-3580975</t>
         </is>
       </c>
       <c r="D2" s="5" t="inlineStr">
         <is>
-          <t>Economia</t>
+          <t>Mundo</t>
         </is>
       </c>
       <c r="E2" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18  7:23 AM</t>
+          <t>2026-08-25  9:21 PM</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/amp/economia/finanzas-personales/estas-son-las-cedulas-que-tienen-que-declarar-renta-esta-semana-del-18-al-21-de-agosto-3578997</t>
+          <t>https://www.eltiempo.com/amp/mundo/venezuela/venezuela-suma-mas-de-un-ano-bajo-estado-de-excepcion-inconstitucional-la-acumulacion-de-competencias-del-ejecutivo-crecio-de-manera-exponencial-3580975</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>La Dian recomienda realizar este proceso antes de que venza el plazo para evitar multas y sanciones.</t>
+          <t>Delcy Rodríguez opera bajo decretos de excepción que eluden controles constitucionales y centralizan el poder y recursos. Informe.</t>
         </is>
       </c>
       <c r="H2" s="9" t="inlineStr">
@@ -788,17 +788,21 @@
         </is>
       </c>
       <c r="I2" s="10" t="n">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="J2" s="8" t="inlineStr">
         <is>
-          <t>muy reciente, tema masivo de economia, tema con traccion de actualidad</t>
-        </is>
-      </c>
-      <c r="K2" s="8" t="inlineStr"/>
+          <t>Refleja la crisis política y la prolongación del estado de excepción, tema de alta relevancia nacional y buscado en buscadores</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>excepción inconstitucional</t>
+        </is>
+      </c>
       <c r="L2" s="11" t="inlineStr">
         <is>
-          <t>Heuristico</t>
+          <t>Groq (openai/gpt-oss-120b)</t>
         </is>
       </c>
     </row>
@@ -806,32 +810,32 @@
       <c r="A3" s="12" t="inlineStr"/>
       <c r="B3" s="13" t="inlineStr">
         <is>
-          <t>Más de 30000 empresas cerraron en Argentina desde la llegada</t>
+          <t>Corte devuelve 9 artículos clave de reforma pensional</t>
         </is>
       </c>
       <c r="C3" s="14" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/mundo/latinoamerica/mas-de-30-000-empresas-cerraron-en-argentina-desde-la-llegada-de-javier-milei-conozca-la-razon-3579007</t>
+          <t>https://www.eltiempo.com/economia/sectores/estos-son-los-nueve-articulos-clave-de-la-reforma-pensional-que-la-corte-devolvio-para-correccion-en-el-congreso-3581065</t>
         </is>
       </c>
       <c r="D3" s="15" t="inlineStr">
         <is>
-          <t>Mundo</t>
+          <t>Economia</t>
         </is>
       </c>
       <c r="E3" s="16" t="inlineStr">
         <is>
-          <t>2026-08-18  8:47 AM</t>
+          <t>2026-08-25  9:12 PM</t>
         </is>
       </c>
       <c r="F3" s="17" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/amp/mundo/latinoamerica/mas-de-30-000-empresas-cerraron-en-argentina-desde-la-llegada-de-javier-milei-conozca-la-razon-3579007</t>
+          <t>https://www.eltiempo.com/amp/economia/sectores/estos-son-los-nueve-articulos-clave-de-la-reforma-pensional-que-la-corte-devolvio-para-correccion-en-el-congreso-3581065</t>
         </is>
       </c>
       <c r="G3" s="18" t="inlineStr">
         <is>
-          <t>La cantidad de empresas se ubicó en 481.724 en mayo, un dato inferior al máximo histórico, que se alcanzó en febrero de 2012 con 540.282 firmas.</t>
+          <t>El paquete de apartados devueltos abarca desde la propiedad de los ahorros hasta beneficios para mujeres y minorías.</t>
         </is>
       </c>
       <c r="H3" s="19" t="inlineStr">
@@ -840,17 +844,21 @@
         </is>
       </c>
       <c r="I3" s="20" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="J3" s="18" t="inlineStr">
         <is>
-          <t>muy reciente, categoria activa: mundo, angulo util para busqueda</t>
-        </is>
-      </c>
-      <c r="K3" s="18" t="inlineStr"/>
+          <t>Alto interés por la reforma pensional y la intervención judicial, tema clave en la agenda económica nacional</t>
+        </is>
+      </c>
+      <c r="K3" s="18" t="inlineStr">
+        <is>
+          <t>reforma pensional</t>
+        </is>
+      </c>
       <c r="L3" s="21" t="inlineStr">
         <is>
-          <t>Heuristico</t>
+          <t>Groq (openai/gpt-oss-120b)</t>
         </is>
       </c>
     </row>
@@ -858,32 +866,32 @@
       <c r="A4" s="2" t="inlineStr"/>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>La OMS analiza la evolución del brote de ébola</t>
+          <t>Turberas: superhéroes del agua contra El Niño</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/salud/la-oms-analiza-la-evolucion-del-brote-de-ebola-en-la-republica-democratica-del-congo-3579018</t>
+          <t>https://www.eltiempo.com/vida/medio-ambiente/las-turberas-el-humedal-con-superpoderes-que-casi-nadie-conoce-y-que-puede-ser-clave-frente-al-fenomeno-de-el-nino-3581046</t>
         </is>
       </c>
       <c r="D4" s="22" t="inlineStr">
         <is>
-          <t>Salud</t>
+          <t>Vida</t>
         </is>
       </c>
       <c r="E4" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18  7:43 AM</t>
+          <t>2026-08-25  7:08 PM</t>
         </is>
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/amp/salud/la-oms-analiza-la-evolucion-del-brote-de-ebola-en-la-republica-democratica-del-congo-3579018</t>
+          <t>https://www.eltiempo.com/amp/vida/medio-ambiente/las-turberas-el-humedal-con-superpoderes-que-casi-nadie-conoce-y-que-puede-ser-clave-frente-al-fenomeno-de-el-nino-3581046</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>De mantenerse el ritmo actual de nuevos casos y fallecimientos, la epidemia podría superar esas cifras a largo plazo.</t>
+          <t>Las turberas están en páramos, morichales, selvas y otros humedales. Pueden almacenar enormes cantidades de agua y carbono.</t>
         </is>
       </c>
       <c r="H4" s="9" t="inlineStr">
@@ -892,17 +900,21 @@
         </is>
       </c>
       <c r="I4" s="10" t="n">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="J4" s="8" t="inlineStr">
         <is>
-          <t>muy reciente, tema masivo de salud, tema con traccion de actualidad</t>
-        </is>
-      </c>
-      <c r="K4" s="8" t="inlineStr"/>
+          <t>Une palabras clave de alto interés (turberas, El Niño, agua) y destaca su papel ambiental, generando clics y relevancia nacional</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>turberas</t>
+        </is>
+      </c>
       <c r="L4" s="11" t="inlineStr">
         <is>
-          <t>Heuristico</t>
+          <t>Groq (openai/gpt-oss-120b)</t>
         </is>
       </c>
     </row>
@@ -910,32 +922,32 @@
       <c r="A5" s="12" t="inlineStr"/>
       <c r="B5" s="13" t="inlineStr">
         <is>
-          <t>Esta es la esperanza tras el peor terremoto</t>
+          <t>La fortuna millonaria de Dolly Parton</t>
         </is>
       </c>
       <c r="C5" s="14" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/colombia/otras-ciudades/esta-es-la-esperanza-tras-el-peor-terremoto-en-27-anos-en-colombia-historias-imagenes-y-reconstruccion-despues-de-la-tragedia-3578996</t>
+          <t>https://www.eltiempo.com/cultura/gente/de-cuanto-era-la-fortuna-de-dolly-parton-el-millonario-patrimonio-que-dejo-la-reina-del-country-3581027</t>
         </is>
       </c>
       <c r="D5" s="23" t="inlineStr">
         <is>
-          <t>Colombia</t>
+          <t>Cultura</t>
         </is>
       </c>
       <c r="E5" s="16" t="inlineStr">
         <is>
-          <t>2026-08-18  8:59 AM</t>
+          <t>2026-08-25  6:04 PM</t>
         </is>
       </c>
       <c r="F5" s="17" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/amp/colombia/otras-ciudades/esta-es-la-esperanza-tras-el-peor-terremoto-en-27-anos-en-colombia-historias-imagenes-y-reconstruccion-despues-de-la-tragedia-3578996</t>
+          <t>https://www.eltiempo.com/amp/cultura/gente/de-cuanto-era-la-fortuna-de-dolly-parton-el-millonario-patrimonio-que-dejo-la-reina-del-country-3581027</t>
         </is>
       </c>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>Cubrimiento especial de EL TIEMPO en las regiones devastadas por el temblor de 7,4 del lunes 10 de agosto.</t>
+          <t>Dolly Parton dejó una millonaria fortuna construida con música, negocios, regalías y proyectos empresariales</t>
         </is>
       </c>
       <c r="H5" s="19" t="inlineStr">
@@ -944,17 +956,21 @@
         </is>
       </c>
       <c r="I5" s="20" t="n">
-        <v>83</v>
+        <v>92</v>
       </c>
       <c r="J5" s="18" t="inlineStr">
         <is>
-          <t>muy reciente, tema masivo de colombia, tema con traccion de actualidad</t>
-        </is>
-      </c>
-      <c r="K5" s="18" t="inlineStr"/>
+          <t>Alta relevancia por la figura internacional y el interés en su patrimonio, palabras clave fuertes y tendencia de búsquedas</t>
+        </is>
+      </c>
+      <c r="K5" s="18" t="inlineStr">
+        <is>
+          <t>fortuna Dolly Parton</t>
+        </is>
+      </c>
       <c r="L5" s="21" t="inlineStr">
         <is>
-          <t>Heuristico</t>
+          <t>Groq (openai/gpt-oss-120b)</t>
         </is>
       </c>
     </row>
@@ -962,32 +978,32 @@
       <c r="A6" s="2" t="inlineStr"/>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>Un estudio encontró una relación entre la amistad la inteligencia</t>
+          <t>EE.UU. acelera visas B en Bogotá hasta 2026</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/vida/ciencia/un-estudio-encontro-una-relacion-entre-la-amistad-la-inteligencia-y-la-satisfaccion-con-la-vida-3579030</t>
+          <t>https://www.eltiempo.com/bogota/estados-unidos-agiliza-citas-de-visa-b-de-no-inmigrante-en-bogota-conozca-los-requisitos-y-como-funciona-el-programa-3580792</t>
         </is>
       </c>
       <c r="D6" s="24" t="inlineStr">
         <is>
-          <t>Vida</t>
+          <t>Bogota</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18  8:03 AM</t>
+          <t>2026-08-25  9:18 PM</t>
         </is>
       </c>
       <c r="F6" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/amp/vida/ciencia/un-estudio-encontro-una-relacion-entre-la-amistad-la-inteligencia-y-la-satisfaccion-con-la-vida-3579030</t>
+          <t>https://www.eltiempo.com/amp/bogota/estados-unidos-agiliza-citas-de-visa-b-de-no-inmigrante-en-bogota-conozca-los-requisitos-y-como-funciona-el-programa-3580792</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Entre las personas con niveles altos de inteligencia, la relación entre socialización frecuente y satisfacción se invertía, según los resultados.</t>
+          <t>La medida estará disponible en algunas embajadas y consulados de Estados Unidos hasta el 31 de diciembre de 2026.</t>
         </is>
       </c>
       <c r="H6" s="9" t="inlineStr">
@@ -996,17 +1012,21 @@
         </is>
       </c>
       <c r="I6" s="10" t="n">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>muy reciente, categoria activa: vida, tema con traccion de actualidad</t>
-        </is>
-      </c>
-      <c r="K6" s="8" t="inlineStr"/>
+          <t>Alta demanda de visas y relevancia para viajeros y negocios en Colombia</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>visas B Bogotá</t>
+        </is>
+      </c>
       <c r="L6" s="11" t="inlineStr">
         <is>
-          <t>Heuristico</t>
+          <t>Groq (openai/gpt-oss-120b)</t>
         </is>
       </c>
     </row>
@@ -1014,51 +1034,55 @@
       <c r="A7" s="12" t="inlineStr"/>
       <c r="B7" s="13" t="inlineStr">
         <is>
-          <t>Kolthoum Akbari la Viuda Negra de Irán que asesinó</t>
+          <t>Presidente De La Espriella gobernará desde Casa de Nariño</t>
         </is>
       </c>
       <c r="C7" s="14" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/cultura/gente/kolthoum-akbari-la-viuda-negra-de-iran-que-asesino-a-10-de-sus-esposos-durante-dos-decadas-para-quedarse-con-sus-herencias-y-fue-condenada-a-muerte-3579017</t>
+          <t>https://www.eltiempo.com/politica/gobierno/abelardo-de-la-espriella-decidio-que-tambien-gobernara-desde-la-casa-de-narino-equipo-alista-el-palacio-para-su-llegada-3581041</t>
         </is>
       </c>
       <c r="D7" s="25" t="inlineStr">
         <is>
-          <t>Cultura</t>
+          <t>Politica</t>
         </is>
       </c>
       <c r="E7" s="16" t="inlineStr">
         <is>
-          <t>2026-08-18  7:53 AM</t>
+          <t>2026-08-25  9:03 PM</t>
         </is>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/amp/cultura/gente/kolthoum-akbari-la-viuda-negra-de-iran-que-asesino-a-10-de-sus-esposos-durante-dos-decadas-para-quedarse-con-sus-herencias-y-fue-condenada-a-muerte-3579017</t>
+          <t>https://www.eltiempo.com/amp/politica/gobierno/abelardo-de-la-espriella-decidio-que-tambien-gobernara-desde-la-casa-de-narino-equipo-alista-el-palacio-para-su-llegada-3581041</t>
         </is>
       </c>
       <c r="G7" s="18" t="inlineStr">
         <is>
-          <t>Varias de las víctimas habrían recibido sedantes, medicamentos y alcohol antes de morir.</t>
-        </is>
-      </c>
-      <c r="H7" s="26" t="inlineStr">
-        <is>
-          <t>Alto</t>
+          <t>El jefe de Estado estuvo despachando las últimas semanas desde el Palacio de San Carlos, donde funciona la Cancillería.</t>
+        </is>
+      </c>
+      <c r="H7" s="19" t="inlineStr">
+        <is>
+          <t>Muy alto</t>
         </is>
       </c>
       <c r="I7" s="20" t="n">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="J7" s="18" t="inlineStr">
         <is>
-          <t>muy reciente, tema con traccion de actualidad, angulo util para busqueda</t>
-        </is>
-      </c>
-      <c r="K7" s="18" t="inlineStr"/>
+          <t>Tema de alta relevancia política nacional y cambio de sede presidencial genera gran interés de búsqueda</t>
+        </is>
+      </c>
+      <c r="K7" s="18" t="inlineStr">
+        <is>
+          <t>Casa de Nariño</t>
+        </is>
+      </c>
       <c r="L7" s="21" t="inlineStr">
         <is>
-          <t>Heuristico</t>
+          <t>Groq (openai/gpt-oss-120b)</t>
         </is>
       </c>
     </row>
@@ -1066,51 +1090,55 @@
       <c r="A8" s="2" t="inlineStr"/>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>Ana Lucía Pineda primera dama de Colombia defendió al ministro</t>
+          <t>Tolima pierde y queda fuera de la Libertadores</t>
         </is>
       </c>
       <c r="C8" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/politica/gobierno/ana-lucia-pineda-primera-dama-de-colombia-defendio-al-ministro-de-vivienda-jaime-andres-beltran-por-supuesto-viaje-a-santa-marta-siga-adelante-3579003</t>
-        </is>
-      </c>
-      <c r="D8" s="27" t="inlineStr">
-        <is>
-          <t>Politica</t>
+          <t>https://www.eltiempo.com/deportes/futbol-internacional/deportes-tolima-busca-la-remontada-contra-independiente-del-valle-en-la-copa-libertadores-minuto-a-minuto-3581044</t>
+        </is>
+      </c>
+      <c r="D8" s="26" t="inlineStr">
+        <is>
+          <t>Deportes</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18  8:05 AM</t>
+          <t>2026-08-25  9:26 PM</t>
         </is>
       </c>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/amp/politica/gobierno/ana-lucia-pineda-primera-dama-de-colombia-defendio-al-ministro-de-vivienda-jaime-andres-beltran-por-supuesto-viaje-a-santa-marta-siga-adelante-3579003</t>
+          <t>https://www.eltiempo.com/amp/deportes/futbol-internacional/deportes-tolima-busca-la-remontada-contra-independiente-del-valle-en-la-copa-libertadores-minuto-a-minuto-3581044</t>
         </is>
       </c>
       <c r="G8" s="8" t="inlineStr">
         <is>
-          <t>El jefe de esta cartera fue visto en una playa de esta ciudad en medio de la emergencia por el terremoto del pasado 10 de agosto.</t>
-        </is>
-      </c>
-      <c r="H8" s="28" t="inlineStr">
+          <t>El partido se jugó en el estadio Banco Guayaquil, en Quito.</t>
+        </is>
+      </c>
+      <c r="H8" s="27" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
       <c r="I8" s="10" t="n">
-        <v>73</v>
+        <v>85</v>
       </c>
       <c r="J8" s="8" t="inlineStr">
         <is>
-          <t>muy reciente, tema masivo de politica, tema con traccion de actualidad</t>
-        </is>
-      </c>
-      <c r="K8" s="8" t="inlineStr"/>
+          <t>Incluye palabras clave de alto búsqueda como Tolima, Libertadores y derrota, atrayendo a lectores deportivos nacionales</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>Tolima Libertadores</t>
+        </is>
+      </c>
       <c r="L8" s="11" t="inlineStr">
         <is>
-          <t>Heuristico</t>
+          <t>Groq (openai/gpt-oss-120b)</t>
         </is>
       </c>
     </row>
@@ -1118,51 +1146,55 @@
       <c r="A9" s="12" t="inlineStr"/>
       <c r="B9" s="13" t="inlineStr">
         <is>
-          <t>Identidad de la mujer que cayó al embalse de Tominé</t>
+          <t>Corte salva reforma pensional, devuelve nueve artículos</t>
         </is>
       </c>
       <c r="C9" s="14" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/bogota/esta-es-la-identidad-de-la-mujer-que-cayo-al-embalse-de-tomine-en-guatavita-cundinamarca-luego-de-un-accidente-entre-dos-lanchas-esto-se-sabe-3579016</t>
-        </is>
-      </c>
-      <c r="D9" s="29" t="inlineStr">
-        <is>
-          <t>Bogota</t>
+          <t>https://www.eltiempo.com/justicia/cortes/urgente-corte-constitucional-salvo-la-reforma-pensional-pero-devolvio-por-tramite-nueve-articulos-al-congreso-3580994</t>
+        </is>
+      </c>
+      <c r="D9" s="28" t="inlineStr">
+        <is>
+          <t>Justicia</t>
         </is>
       </c>
       <c r="E9" s="16" t="inlineStr">
         <is>
-          <t>2026-08-18  8:30 AM</t>
+          <t>2026-08-25  9:25 PM</t>
         </is>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/amp/bogota/esta-es-la-identidad-de-la-mujer-que-cayo-al-embalse-de-tomine-en-guatavita-cundinamarca-luego-de-un-accidente-entre-dos-lanchas-esto-se-sabe-3579016</t>
+          <t>https://www.eltiempo.com/amp/justicia/cortes/urgente-corte-constitucional-salvo-la-reforma-pensional-pero-devolvio-por-tramite-nueve-articulos-al-congreso-3580994</t>
         </is>
       </c>
       <c r="G9" s="18" t="inlineStr">
         <is>
-          <t>En la nave afectada viajaban cinco ocupantes: cuatro adultos y un menor de edad.</t>
-        </is>
-      </c>
-      <c r="H9" s="26" t="inlineStr">
+          <t>Entre los artículos que salvó está la ventana de oportunidad, que permitió el traslado de régimen.</t>
+        </is>
+      </c>
+      <c r="H9" s="29" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
       <c r="I9" s="20" t="n">
-        <v>71</v>
+        <v>85</v>
       </c>
       <c r="J9" s="18" t="inlineStr">
         <is>
-          <t>muy reciente, categoria activa: bogota, tema con traccion de actualidad</t>
-        </is>
-      </c>
-      <c r="K9" s="18" t="inlineStr"/>
+          <t>Combina términos de alta relevancia (Corte Constitucional, reforma pensional) con acción clara, generando clics y posicionamiento en búsqued</t>
+        </is>
+      </c>
+      <c r="K9" s="18" t="inlineStr">
+        <is>
+          <t>reforma pensional</t>
+        </is>
+      </c>
       <c r="L9" s="21" t="inlineStr">
         <is>
-          <t>Heuristico</t>
+          <t>Groq (openai/gpt-oss-120b)</t>
         </is>
       </c>
     </row>
@@ -1170,51 +1202,55 @@
       <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Así operaba la red señalada de asaltar golpear y agredir</t>
+          <t>Buenaventura relanza turismo de ballenas tras sismo</t>
         </is>
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/justicia/delitos/asi-operaba-la-red-senalada-de-asaltar-golpear-y-agredir-sexualmente-a-sus-victimas-en-la-via-cartagena-baru-3579019</t>
+          <t>https://www.eltiempo.com/colombia/cali/de-la-tragedia-a-la-reactivacion-buenaventura-abre-sus-puertas-al-turismo-de-ballenas-yubartas-tras-el-sismo-3581058</t>
         </is>
       </c>
       <c r="D10" s="30" t="inlineStr">
         <is>
-          <t>Justicia</t>
+          <t>Colombia</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>2026-08-18  7:48 AM</t>
+          <t>2026-08-25  7:47 PM</t>
         </is>
       </c>
       <c r="F10" s="7" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/amp/justicia/delitos/asi-operaba-la-red-senalada-de-asaltar-golpear-y-agredir-sexualmente-a-sus-victimas-en-la-via-cartagena-baru-3579019</t>
+          <t>https://www.eltiempo.com/amp/colombia/cali/de-la-tragedia-a-la-reactivacion-buenaventura-abre-sus-puertas-al-turismo-de-ballenas-yubartas-tras-el-sismo-3581058</t>
         </is>
       </c>
       <c r="G10" s="8" t="inlineStr">
         <is>
-          <t>El grupo estaría relacionado con al menos dos hechos ocurridos el 22 de febrero y el 3 de marzo de 2025, en el corregimiento de Pasacaballos.</t>
-        </is>
-      </c>
-      <c r="H10" s="28" t="inlineStr">
+          <t>La iniciativa busca dinamizar la economía local y respaldar la recuperación del Pacífico vallecaucano tras las afectaciones por el terremoto.</t>
+        </is>
+      </c>
+      <c r="H10" s="27" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
       <c r="I10" s="10" t="n">
-        <v>67</v>
+        <v>85</v>
       </c>
       <c r="J10" s="8" t="inlineStr">
         <is>
-          <t>muy reciente, categoria activa: justicia</t>
-        </is>
-      </c>
-      <c r="K10" s="8" t="inlineStr"/>
+          <t>Combina palabras clave de turismo, Buenaventura y sismo, atrayendo búsquedas locales y de recuperación económica</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>turismo de ballenas Buenaventura</t>
+        </is>
+      </c>
       <c r="L10" s="11" t="inlineStr">
         <is>
-          <t>Heuristico</t>
+          <t>Groq (openai/gpt-oss-120b)</t>
         </is>
       </c>
     </row>
@@ -1222,51 +1258,55 @@
       <c r="A11" s="12" t="inlineStr"/>
       <c r="B11" s="13" t="inlineStr">
         <is>
-          <t>Diego Simeone acabó con la novela de Julián Álvarez</t>
+          <t>Celular antes de dormir daña tu visión</t>
         </is>
       </c>
       <c r="C11" s="14" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/deportes/futbol-internacional/diego-simeone-acabo-con-la-novela-de-julian-alvarez-tajantes-declaraciones-tras-la-opcion-de-irse-del-atletico-de-madrid-3579039</t>
+          <t>https://www.eltiempo.com/salud/jorge-pradas-oftalmologo-advierte-sobre-usar-el-celular-antes-de-dormir-es-como-apuntar-una-linterna-directamente-a-tu-ojo-en-la-oscuridad-3580948</t>
         </is>
       </c>
       <c r="D11" s="31" t="inlineStr">
         <is>
-          <t>Deportes</t>
+          <t>Salud</t>
         </is>
       </c>
       <c r="E11" s="16" t="inlineStr">
         <is>
-          <t>2026-08-18  8:58 AM</t>
+          <t>2026-08-25  1:54 PM</t>
         </is>
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>https://www.eltiempo.com/amp/deportes/futbol-internacional/diego-simeone-acabo-con-la-novela-de-julian-alvarez-tajantes-declaraciones-tras-la-opcion-de-irse-del-atletico-de-madrid-3579039</t>
+          <t>https://www.eltiempo.com/amp/salud/jorge-pradas-oftalmologo-advierte-sobre-usar-el-celular-antes-de-dormir-es-como-apuntar-una-linterna-directamente-a-tu-ojo-en-la-oscuridad-3580948</t>
         </is>
       </c>
       <c r="G11" s="18" t="inlineStr">
         <is>
-          <t>El argentino se quedará en el equipo.</t>
-        </is>
-      </c>
-      <c r="H11" s="26" t="inlineStr">
+          <t>Lo que ocurre con la pupila en un ambiente completamente oscuro y señaló que este hábito puede estar relacionado con fatiga visual.</t>
+        </is>
+      </c>
+      <c r="H11" s="29" t="inlineStr">
         <is>
           <t>Alto</t>
         </is>
       </c>
       <c r="I11" s="20" t="n">
-        <v>65</v>
+        <v>85</v>
       </c>
       <c r="J11" s="18" t="inlineStr">
         <is>
-          <t>muy reciente, categoria activa: deportes, angulo util para busqueda</t>
-        </is>
-      </c>
-      <c r="K11" s="18" t="inlineStr"/>
+          <t>Alta relevancia por salud visual y hábito digital, genera gran interés y búsquedas</t>
+        </is>
+      </c>
+      <c r="K11" s="18" t="inlineStr">
+        <is>
+          <t>celular antes de dormir</t>
+        </is>
+      </c>
       <c r="L11" s="21" t="inlineStr">
         <is>
-          <t>Heuristico</t>
+          <t>Groq (openai/gpt-oss-120b)</t>
         </is>
       </c>
     </row>

</xml_diff>